<commit_message>
Updates made on 17Sep26updates branch
</commit_message>
<xml_diff>
--- a/Talent360i_Output.xlsx
+++ b/Talent360i_Output.xlsx
@@ -1041,7 +1041,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1443,6 +1443,131 @@
       <c r="E16" t="inlineStr">
         <is>
           <t>2026-09-11T12:02:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>ASG-20260917135151435635</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Q-0043</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Skip documentation to meet speed targets and update records after the close cycle.</t>
+        </is>
+      </c>
+      <c r="D17" t="b">
+        <v>0</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2026-09-17T13:52:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>ASG-20260917135151435635</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Q-0046</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Resolve the item informally without linking the action to controls, metrics or evidence.</t>
+        </is>
+      </c>
+      <c r="D18" t="b">
+        <v>0</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2026-09-17T13:52:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>ASG-20260917135151435635</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Q-0047</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Apply the SOP, maintain evidence, escalate exceptions, and document the rationale for AP Reconciliations (Subledger/GL, Vendor Statements).</t>
+        </is>
+      </c>
+      <c r="D19" t="b">
+        <v>1</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2026-09-17T13:52:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>ASG-20260917135151435635</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Q-0049</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Follow the standard SOP only when instructed and wait for review before taking action.</t>
+        </is>
+      </c>
+      <c r="D20" t="b">
+        <v>0</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2026-09-17T13:52:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>ASG-20260917135151435635</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Q-0050</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Apply the SOP, maintain evidence, escalate exceptions, and document the rationale for Ownership &amp; Delivery.</t>
+        </is>
+      </c>
+      <c r="D21" t="b">
+        <v>1</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2026-09-17T13:52:48</t>
         </is>
       </c>
     </row>
@@ -1457,7 +1582,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1725,6 +1850,72 @@
         </is>
       </c>
       <c r="N4" t="inlineStr">
+        <is>
+          <t>Application-calculated result awaiting calibration</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>RST-20260917135248973504</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Application-created record</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ASG-20260917135151435635</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>SYN-U017</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>AP_p2p_senior_associate</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>BP-005</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>SCH-005</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>40</v>
+      </c>
+      <c r="I5" t="n">
+        <v>75</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>2</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Calibrated</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
         <is>
           <t>Application-calculated result awaiting calibration</t>
         </is>
@@ -1741,7 +1932,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1987,6 +2178,64 @@
       <c r="L4" t="inlineStr">
         <is>
           <t>RST-20260911120241582044</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>USA-20260917135315504185</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Application-created record</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>SYN-U017</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>AP_p2p_senior_associate</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>AP_invoice_processing_po_non_po</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Invoice Processing (PO &amp; Non-PO)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Invoice Processing (PO &amp; Non-PO)</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>3</v>
+      </c>
+      <c r="I5" t="n">
+        <v>2</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Assessed</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Calibrated</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>RST-20260917135248973504</t>
         </is>
       </c>
     </row>
@@ -2001,7 +2250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:O5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2141,6 +2390,8 @@
           <t>Assign mapped microlearning / scenario lab and reassess</t>
         </is>
       </c>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2202,6 +2453,8 @@
           <t>Assign mapped microlearning / scenario lab and reassess</t>
         </is>
       </c>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2263,6 +2516,71 @@
           <t>Assign mapped microlearning / scenario lab and reassess</t>
         </is>
       </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>GAP-20260917135316179340</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Application-created record</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>SYN-U017</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>AP_p2p_senior_associate</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>AP_invoice_processing_po_non_po</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Invoice Processing (PO &amp; Non-PO)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Invoice Processing (PO &amp; Non-PO)</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>3</v>
+      </c>
+      <c r="I5" t="n">
+        <v>2</v>
+      </c>
+      <c r="J5" t="n">
+        <v>1</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>TRN-0008</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Assign mapped microlearning / scenario lab and reassess</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2639,7 +2957,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3046,6 +3364,51 @@
       <c r="I9" t="inlineStr">
         <is>
           <t>2026-09-11T12:01:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>REQ-20260917135108456956</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>SYN-U017</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>AP_p2p_senior_associate</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>P2P Senior Associate</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>AP_close_activities_accruals_cutoff_gr_ir</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Close Activities (Accruals, Cutoff, GR/IR)</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>2</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Assigned</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-09-17T13:51:08</t>
         </is>
       </c>
     </row>
@@ -3060,7 +3423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3393,6 +3756,43 @@
       <c r="G9" t="inlineStr">
         <is>
           <t>2026-09-11T12:01:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>AUD-20260917135108456956</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>assessment_request</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>REQ-20260917135108456956</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>SYN-U017</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Skill=Close Activities (Accruals, Cutoff, GR/IR), Level=2</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2026-09-17T13:51:09</t>
         </is>
       </c>
     </row>
@@ -18639,7 +19039,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19001,6 +19401,58 @@
         </is>
       </c>
       <c r="J7" t="inlineStr">
+        <is>
+          <t>Created from approved question bank</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ASG-20260917135151435635</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Application-created record</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>SYN-U017</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>AP_p2p_senior_associate</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>BP-005</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>SCH-005</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
         <is>
           <t>Created from approved question bank</t>
         </is>
@@ -19017,7 +19469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:B36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19392,6 +19844,66 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>ASG-20260917135151435635</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Q-0043</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>ASG-20260917135151435635</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Q-0046</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>ASG-20260917135151435635</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Q-0050</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>ASG-20260917135151435635</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Q-0047</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>ASG-20260917135151435635</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Q-0049</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
added the feature where sme can update the question text
</commit_message>
<xml_diff>
--- a/Talent360i_Output.xlsx
+++ b/Talent360i_Output.xlsx
@@ -3816,7 +3816,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4403,6 +4403,96 @@
       <c r="I13" t="inlineStr">
         <is>
           <t>2026-09-18T15:39:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>REQ-20260918195804693255</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>SYN-U031</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>O2C_associate_revenue_controller</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Associate Revenue Controller</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>O2C_invoicing_standard_complex</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Invoicing (Standard/Complex)</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>5</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Requested</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-09-18T19:58:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>REQ-20260918200042515999</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>SYN-U017</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>AP_p2p_senior_associate</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>P2P Senior Associate</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>AP_tax_withholding_regulatory_basics</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Tax / Withholding &amp; Regulatory Basics</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>5</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Assigned</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-09-18T20:00:42</t>
         </is>
       </c>
     </row>
@@ -4417,7 +4507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4898,6 +4988,80 @@
       <c r="G13" t="inlineStr">
         <is>
           <t>2026-09-18T15:39:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>AUD-20260918195804693255</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>assessment_request</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>REQ-20260918195804693255</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>SYN-U031</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Skill=Invoicing (Standard/Complex), Level=5</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-09-18T19:58:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>AUD-20260918200042515999</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>assessment_request</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>REQ-20260918200042515999</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>SYN-U017</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Skill=Tax / Withholding &amp; Regulatory Basics, Level=5</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2026-09-18T20:00:43</t>
         </is>
       </c>
     </row>
@@ -4912,7 +5076,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N191"/>
+  <dimension ref="A1:N201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16794,6 +16958,656 @@
       <c r="M191" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>REV-20260918200726762812</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Application-created record</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Q-AI-20260918200427929257</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>BP-005</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>AP_p2p_senior_associate</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>AP_tax_withholding_regulatory_basics</t>
+        </is>
+      </c>
+      <c r="G192" t="n">
+        <v>1</v>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>Approve</t>
+        </is>
+      </c>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>Approved for schedule</t>
+        </is>
+      </c>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="L192" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="M192" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>REV-20260918200728879604</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Application-created record</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Q-AI-20260918200429777983</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>BP-005</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>AP_p2p_senior_associate</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>AP_tax_withholding_regulatory_basics</t>
+        </is>
+      </c>
+      <c r="G193" t="n">
+        <v>1</v>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>Approve</t>
+        </is>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>Approved for schedule</t>
+        </is>
+      </c>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="L193" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="M193" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>REV-20260918200730422617</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Application-created record</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Q-AI-20260918200424458847</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>BP-005</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>AP_p2p_senior_associate</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>AP_tax_withholding_regulatory_basics</t>
+        </is>
+      </c>
+      <c r="G194" t="n">
+        <v>1</v>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>Approve</t>
+        </is>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>Approved for schedule</t>
+        </is>
+      </c>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="L194" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="M194" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>REV-20260918200732341078</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Application-created record</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Q-AI-20260918200422336284</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>BP-005</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>AP_p2p_senior_associate</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>AP_tax_withholding_regulatory_basics</t>
+        </is>
+      </c>
+      <c r="G195" t="n">
+        <v>1</v>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>Approve</t>
+        </is>
+      </c>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>Approved for schedule</t>
+        </is>
+      </c>
+      <c r="K195" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="L195" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="M195" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>REV-20260918200734247530</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Application-created record</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Q-AI-20260918200426383004</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>BP-005</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>AP_p2p_senior_associate</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>AP_tax_withholding_regulatory_basics</t>
+        </is>
+      </c>
+      <c r="G196" t="n">
+        <v>1</v>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>Approve</t>
+        </is>
+      </c>
+      <c r="J196" t="inlineStr">
+        <is>
+          <t>Approved for schedule</t>
+        </is>
+      </c>
+      <c r="K196" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="L196" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="M196" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>REV-20260918200736276243</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Application-created record</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Q-AI-20260918200427176463</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>BP-005</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>AP_p2p_senior_associate</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>AP_tax_withholding_regulatory_basics</t>
+        </is>
+      </c>
+      <c r="G197" t="n">
+        <v>1</v>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>Approve</t>
+        </is>
+      </c>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>Approved for schedule</t>
+        </is>
+      </c>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="L197" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="M197" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>REV-20260918200738075741</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Application-created record</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Q-AI-20260918200425294369</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>BP-005</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>AP_p2p_senior_associate</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>AP_tax_withholding_regulatory_basics</t>
+        </is>
+      </c>
+      <c r="G198" t="n">
+        <v>1</v>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>Approve</t>
+        </is>
+      </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>Approved for schedule</t>
+        </is>
+      </c>
+      <c r="K198" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="L198" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="M198" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>REV-20260918200739966214</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Application-created record</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Q-AI-20260918200428944879</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>BP-005</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>AP_p2p_senior_associate</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>AP_tax_withholding_regulatory_basics</t>
+        </is>
+      </c>
+      <c r="G199" t="n">
+        <v>1</v>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>Approve</t>
+        </is>
+      </c>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>Approved for schedule</t>
+        </is>
+      </c>
+      <c r="K199" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="L199" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="M199" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>REV-20260918200741799433</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Application-created record</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Q-AI-20260918200421585636</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>BP-005</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>AP_p2p_senior_associate</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>AP_tax_withholding_regulatory_basics</t>
+        </is>
+      </c>
+      <c r="G200" t="n">
+        <v>1</v>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>Approve</t>
+        </is>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>Approved for schedule</t>
+        </is>
+      </c>
+      <c r="K200" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="L200" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="M200" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>REV-20260918200744869089</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Application-created record</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Q-AI-20260918200423635576</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>BP-005</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>AP_p2p_senior_associate</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>AP_tax_withholding_regulatory_basics</t>
+        </is>
+      </c>
+      <c r="G201" t="n">
+        <v>1</v>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>Needs Revision</t>
+        </is>
+      </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>Rewrite</t>
+        </is>
+      </c>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t>Rewrite required</t>
+        </is>
+      </c>
+      <c r="K201" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="L201" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="M201" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -16808,7 +17622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA141"/>
+  <dimension ref="A1:AB151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16934,15 +17748,20 @@
       </c>
       <c r="Y1" t="inlineStr">
         <is>
+          <t>ready_for_schedule</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
           <t>source_question_reference</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>ai_confidence</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>schedule_scope</t>
         </is>
@@ -33686,6 +34505,1236 @@
         <is>
           <t>Requires SME approval before scheduling</t>
         </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Q-AI-20260918200421585636</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>BP-005</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Application-created SME wording override</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>AP_p2p_senior_associate</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>P2P Senior Associate</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>AP_tax_withholding_regulatory_basics</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>Tax / Withholding &amp; Regulatory Basics</t>
+        </is>
+      </c>
+      <c r="I142" t="n">
+        <v>5</v>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>AI-generated from role and skill definition</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>Multiple Choice - Scenario</t>
+        </is>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>What is the main purpose of withholding tax?</t>
+        </is>
+      </c>
+      <c r="M142" t="inlineStr">
+        <is>
+          <t>To increase the overall tax rate</t>
+        </is>
+      </c>
+      <c r="N142" t="inlineStr">
+        <is>
+          <t>To ensure tax revenue is collected in advance</t>
+        </is>
+      </c>
+      <c r="O142" t="inlineStr">
+        <is>
+          <t>To reduce tax liability for corporations</t>
+        </is>
+      </c>
+      <c r="P142" t="inlineStr">
+        <is>
+          <t>To provide tax benefits for nonprofit organizations</t>
+        </is>
+      </c>
+      <c r="Q142" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="R142" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S142" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="T142" t="inlineStr">
+        <is>
+          <t>Pending SME Review</t>
+        </is>
+      </c>
+      <c r="U142" t="inlineStr">
+        <is>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="V142" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W142" t="inlineStr">
+        <is>
+          <t>{"skill": "Tax / Withholding &amp; Regulatory Basics", "level": 5}</t>
+        </is>
+      </c>
+      <c r="X142" t="inlineStr">
+        <is>
+          <t>Requires SME approval before scheduling</t>
+        </is>
+      </c>
+      <c r="Y142" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Q-AI-20260918200422336284</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>BP-005</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Application-created SME wording override</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>AP_p2p_senior_associate</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>P2P Senior Associate</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>AP_tax_withholding_regulatory_basics</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>Tax / Withholding &amp; Regulatory Basics</t>
+        </is>
+      </c>
+      <c r="I143" t="n">
+        <v>5</v>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>AI-generated from role and skill definition</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>Multiple Choice - Scenario</t>
+        </is>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>Which of the following is typically subject to withholding tax?</t>
+        </is>
+      </c>
+      <c r="M143" t="inlineStr">
+        <is>
+          <t>Interest income from savings accounts</t>
+        </is>
+      </c>
+      <c r="N143" t="inlineStr">
+        <is>
+          <t>Rental income from property</t>
+        </is>
+      </c>
+      <c r="O143" t="inlineStr">
+        <is>
+          <t>Wages paid to employees</t>
+        </is>
+      </c>
+      <c r="P143" t="inlineStr">
+        <is>
+          <t>Capital gains from stock sales</t>
+        </is>
+      </c>
+      <c r="Q143" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="R143" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S143" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="T143" t="inlineStr">
+        <is>
+          <t>Pending SME Review</t>
+        </is>
+      </c>
+      <c r="U143" t="inlineStr">
+        <is>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="V143" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W143" t="inlineStr">
+        <is>
+          <t>{"skill": "Tax / Withholding &amp; Regulatory Basics", "level": 5}</t>
+        </is>
+      </c>
+      <c r="X143" t="inlineStr">
+        <is>
+          <t>Requires SME approval before scheduling</t>
+        </is>
+      </c>
+      <c r="Y143" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Q-AI-20260918200423635576</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>BP-005</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Application-created SME wording override</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>AP_p2p_senior_associate</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>P2P Senior Associate</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>AP_tax_withholding_regulatory_basics</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>Tax / Withholding &amp; Regulatory Basics</t>
+        </is>
+      </c>
+      <c r="I144" t="n">
+        <v>5</v>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>AI-generated from role and skill definition</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>Multiple Choice - Scenario</t>
+        </is>
+      </c>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t>What form is used by employees to indicate their tax withholding preferences?</t>
+        </is>
+      </c>
+      <c r="M144" t="inlineStr">
+        <is>
+          <t>Form W-2</t>
+        </is>
+      </c>
+      <c r="N144" t="inlineStr">
+        <is>
+          <t>Form 1099</t>
+        </is>
+      </c>
+      <c r="O144" t="inlineStr">
+        <is>
+          <t>Form W-4</t>
+        </is>
+      </c>
+      <c r="P144" t="inlineStr">
+        <is>
+          <t>Form 1040</t>
+        </is>
+      </c>
+      <c r="Q144" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="R144" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S144" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="T144" t="inlineStr">
+        <is>
+          <t>Pending SME Review</t>
+        </is>
+      </c>
+      <c r="U144" t="inlineStr">
+        <is>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="V144" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W144" t="inlineStr">
+        <is>
+          <t>{"skill": "Tax / Withholding &amp; Regulatory Basics", "level": 5}</t>
+        </is>
+      </c>
+      <c r="X144" t="inlineStr">
+        <is>
+          <t>Requires SME approval before scheduling</t>
+        </is>
+      </c>
+      <c r="Y144" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Q-AI-20260918200424458847</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>BP-005</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Application-created SME wording override</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>AP_p2p_senior_associate</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>P2P Senior Associate</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>AP_tax_withholding_regulatory_basics</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>Tax / Withholding &amp; Regulatory Basics</t>
+        </is>
+      </c>
+      <c r="I145" t="n">
+        <v>5</v>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>AI-generated from role and skill definition</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>Multiple Choice - Scenario</t>
+        </is>
+      </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>What is the maximum percentage of an employee's paycheck that can be withheld for federal income tax?</t>
+        </is>
+      </c>
+      <c r="M145" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="N145" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="O145" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="P145" t="inlineStr">
+        <is>
+          <t>There is no maximum percentage</t>
+        </is>
+      </c>
+      <c r="Q145" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="R145" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S145" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="T145" t="inlineStr">
+        <is>
+          <t>Pending SME Review</t>
+        </is>
+      </c>
+      <c r="U145" t="inlineStr">
+        <is>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="V145" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W145" t="inlineStr">
+        <is>
+          <t>{"skill": "Tax / Withholding &amp; Regulatory Basics", "level": 5}</t>
+        </is>
+      </c>
+      <c r="X145" t="inlineStr">
+        <is>
+          <t>Requires SME approval before scheduling</t>
+        </is>
+      </c>
+      <c r="Y145" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Q-AI-20260918200425294369</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>BP-005</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Application-created SME wording override</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>AP_p2p_senior_associate</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>P2P Senior Associate</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>AP_tax_withholding_regulatory_basics</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>Tax / Withholding &amp; Regulatory Basics</t>
+        </is>
+      </c>
+      <c r="I146" t="n">
+        <v>5</v>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>AI-generated from role and skill definition</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>Multiple Choice - Scenario</t>
+        </is>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>Which of the following is a common consequence of failing to withhold the correct amount of tax?</t>
+        </is>
+      </c>
+      <c r="M146" t="inlineStr">
+        <is>
+          <t>Increased tax refund</t>
+        </is>
+      </c>
+      <c r="N146" t="inlineStr">
+        <is>
+          <t>Penalties and interest charges</t>
+        </is>
+      </c>
+      <c r="O146" t="inlineStr">
+        <is>
+          <t>Lower tax liability in the following year</t>
+        </is>
+      </c>
+      <c r="P146" t="inlineStr">
+        <is>
+          <t>No significant impact</t>
+        </is>
+      </c>
+      <c r="Q146" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="R146" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S146" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="T146" t="inlineStr">
+        <is>
+          <t>Pending SME Review</t>
+        </is>
+      </c>
+      <c r="U146" t="inlineStr">
+        <is>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="V146" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W146" t="inlineStr">
+        <is>
+          <t>{"skill": "Tax / Withholding &amp; Regulatory Basics", "level": 5}</t>
+        </is>
+      </c>
+      <c r="X146" t="inlineStr">
+        <is>
+          <t>Requires SME approval before scheduling</t>
+        </is>
+      </c>
+      <c r="Y146" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Q-AI-20260918200426383004</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>BP-005</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Application-created SME wording override</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>AP_p2p_senior_associate</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>P2P Senior Associate</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>AP_tax_withholding_regulatory_basics</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>Tax / Withholding &amp; Regulatory Basics</t>
+        </is>
+      </c>
+      <c r="I147" t="n">
+        <v>5</v>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>AI-generated from role and skill definition</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>Multiple Choice - Scenario</t>
+        </is>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>What is the primary purpose of the IRS Form 941?</t>
+        </is>
+      </c>
+      <c r="M147" t="inlineStr">
+        <is>
+          <t>To report annual income tax returns</t>
+        </is>
+      </c>
+      <c r="N147" t="inlineStr">
+        <is>
+          <t>To report quarterly payroll taxes</t>
+        </is>
+      </c>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t>To claim tax credits for businesses</t>
+        </is>
+      </c>
+      <c r="P147" t="inlineStr">
+        <is>
+          <t>To notify the IRS of a business closure</t>
+        </is>
+      </c>
+      <c r="Q147" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="R147" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S147" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="T147" t="inlineStr">
+        <is>
+          <t>Pending SME Review</t>
+        </is>
+      </c>
+      <c r="U147" t="inlineStr">
+        <is>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="V147" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W147" t="inlineStr">
+        <is>
+          <t>{"skill": "Tax / Withholding &amp; Regulatory Basics", "level": 5}</t>
+        </is>
+      </c>
+      <c r="X147" t="inlineStr">
+        <is>
+          <t>Requires SME approval before scheduling</t>
+        </is>
+      </c>
+      <c r="Y147" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Q-AI-20260918200427176463</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>BP-005</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Application-created SME wording override</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>AP_p2p_senior_associate</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>P2P Senior Associate</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>AP_tax_withholding_regulatory_basics</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>Tax / Withholding &amp; Regulatory Basics</t>
+        </is>
+      </c>
+      <c r="I148" t="n">
+        <v>5</v>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>AI-generated from role and skill definition</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>Multiple Choice - Scenario</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>Which of the following types of income is generally exempt from withholding tax?</t>
+        </is>
+      </c>
+      <c r="M148" t="inlineStr">
+        <is>
+          <t>Wages</t>
+        </is>
+      </c>
+      <c r="N148" t="inlineStr">
+        <is>
+          <t>Dividends</t>
+        </is>
+      </c>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>Interest from municipal bonds</t>
+        </is>
+      </c>
+      <c r="P148" t="inlineStr">
+        <is>
+          <t>Bonuses</t>
+        </is>
+      </c>
+      <c r="Q148" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="R148" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S148" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="T148" t="inlineStr">
+        <is>
+          <t>Pending SME Review</t>
+        </is>
+      </c>
+      <c r="U148" t="inlineStr">
+        <is>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="V148" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W148" t="inlineStr">
+        <is>
+          <t>{"skill": "Tax / Withholding &amp; Regulatory Basics", "level": 5}</t>
+        </is>
+      </c>
+      <c r="X148" t="inlineStr">
+        <is>
+          <t>Requires SME approval before scheduling</t>
+        </is>
+      </c>
+      <c r="Y148" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Q-AI-20260918200427929257</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>BP-005</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Application-created SME wording override</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>AP_p2p_senior_associate</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>P2P Senior Associate</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>AP_tax_withholding_regulatory_basics</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>Tax / Withholding &amp; Regulatory Basics</t>
+        </is>
+      </c>
+      <c r="I149" t="n">
+        <v>5</v>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>AI-generated from role and skill definition</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>Multiple Choice - Scenario</t>
+        </is>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>What is a 1099 form used for?</t>
+        </is>
+      </c>
+      <c r="M149" t="inlineStr">
+        <is>
+          <t>To report wages paid to employees</t>
+        </is>
+      </c>
+      <c r="N149" t="inlineStr">
+        <is>
+          <t>To report miscellaneous income not subject to withholding</t>
+        </is>
+      </c>
+      <c r="O149" t="inlineStr">
+        <is>
+          <t>To report tax credits received</t>
+        </is>
+      </c>
+      <c r="P149" t="inlineStr">
+        <is>
+          <t>To report business expenses</t>
+        </is>
+      </c>
+      <c r="Q149" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="R149" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S149" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="T149" t="inlineStr">
+        <is>
+          <t>Pending SME Review</t>
+        </is>
+      </c>
+      <c r="U149" t="inlineStr">
+        <is>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="V149" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W149" t="inlineStr">
+        <is>
+          <t>{"skill": "Tax / Withholding &amp; Regulatory Basics", "level": 5}</t>
+        </is>
+      </c>
+      <c r="X149" t="inlineStr">
+        <is>
+          <t>Requires SME approval before scheduling</t>
+        </is>
+      </c>
+      <c r="Y149" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Q-AI-20260918200428944879</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>BP-005</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Application-created SME wording override</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>AP_p2p_senior_associate</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>P2P Senior Associate</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>AP_tax_withholding_regulatory_basics</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>Tax / Withholding &amp; Regulatory Basics</t>
+        </is>
+      </c>
+      <c r="I150" t="n">
+        <v>5</v>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>AI-generated from role and skill definition</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>Multiple Choice - Scenario</t>
+        </is>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>In the context of tax withholding, what does the term 'FICA' stand for?</t>
+        </is>
+      </c>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>Federal Income Contribution Act</t>
+        </is>
+      </c>
+      <c r="N150" t="inlineStr">
+        <is>
+          <t>Federal Insurance Contributions Act</t>
+        </is>
+      </c>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t>Federal Income Compensation Act</t>
+        </is>
+      </c>
+      <c r="P150" t="inlineStr">
+        <is>
+          <t>Federal Insurance Collection Act</t>
+        </is>
+      </c>
+      <c r="Q150" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="R150" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S150" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="T150" t="inlineStr">
+        <is>
+          <t>Pending SME Review</t>
+        </is>
+      </c>
+      <c r="U150" t="inlineStr">
+        <is>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="V150" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W150" t="inlineStr">
+        <is>
+          <t>{"skill": "Tax / Withholding &amp; Regulatory Basics", "level": 5}</t>
+        </is>
+      </c>
+      <c r="X150" t="inlineStr">
+        <is>
+          <t>Requires SME approval before scheduling</t>
+        </is>
+      </c>
+      <c r="Y150" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Q-AI-20260918200429777983</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>BP-005</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Application-created SME wording override</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>AP</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>AP_p2p_senior_associate</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>P2P Senior Associate</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>AP_tax_withholding_regulatory_basics</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>Tax / Withholding &amp; Regulatory Basics</t>
+        </is>
+      </c>
+      <c r="I151" t="n">
+        <v>5</v>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>AI-generated from role and skill definition</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>Multiple Choice - Scenario</t>
+        </is>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>Which of the following best describes the relationship between withholding tax and estimated tax payments?</t>
+        </is>
+      </c>
+      <c r="M151" t="inlineStr">
+        <is>
+          <t>Withholding tax is always higher than estimated tax payments.</t>
+        </is>
+      </c>
+      <c r="N151" t="inlineStr">
+        <is>
+          <t>Withholding tax is a form of estimated tax payment.</t>
+        </is>
+      </c>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>Estimated tax payments are only for self-employed individuals.</t>
+        </is>
+      </c>
+      <c r="P151" t="inlineStr">
+        <is>
+          <t>There is no relationship between the two.</t>
+        </is>
+      </c>
+      <c r="Q151" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="R151" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S151" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="T151" t="inlineStr">
+        <is>
+          <t>Pending SME Review</t>
+        </is>
+      </c>
+      <c r="U151" t="inlineStr">
+        <is>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="V151" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="W151" t="inlineStr">
+        <is>
+          <t>{"skill": "Tax / Withholding &amp; Regulatory Basics", "level": 5}</t>
+        </is>
+      </c>
+      <c r="X151" t="inlineStr">
+        <is>
+          <t>Requires SME approval before scheduling</t>
+        </is>
+      </c>
+      <c r="Y151" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -33699,7 +35748,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -34271,6 +36320,110 @@
       <c r="J11" t="inlineStr">
         <is>
           <t>you can do better</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ASG-20260918200839942746</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Application-created record</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>SYN-U017</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>AP_p2p_senior_associate</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>BP-005</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>SCH-005</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Created from approved question bank</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ASG-20260918200849618778</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Application-created record</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>SYN-U017</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>AP_p2p_senior_associate</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>BP-005</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>SCH-005</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Created from approved question bank</t>
         </is>
       </c>
     </row>
@@ -34285,7 +36438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B51"/>
+  <dimension ref="A1:B61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -34900,6 +37053,126 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>ASG-20260918200839942746</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Q-AI-20260918200421585636</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>ASG-20260918200839942746</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Q-AI-20260918200424458847</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>ASG-20260918200839942746</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Q-AI-20260918200427176463</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>ASG-20260918200839942746</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Q-AI-20260918200428944879</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>ASG-20260918200839942746</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Q-AI-20260918200429777983</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>ASG-20260918200849618778</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Q-AI-20260918200421585636</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>ASG-20260918200849618778</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Q-AI-20260918200424458847</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>ASG-20260918200849618778</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Q-AI-20260918200427176463</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>ASG-20260918200849618778</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Q-AI-20260918200428944879</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>ASG-20260918200849618778</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Q-AI-20260918200429777983</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>